<commit_message>
Renombrar en Tesoreria la capacidad a Control y tratamiento contable
Peticion del socio: la primera capacidad de Tesoreria pasa de
"Contabilidad y provision fiscal" a "Control y tratamiento contable".

El nombre de la capacidad es la clave de sus objetivos guardados, asi que
cambiarlo solo en el Excel devolvia en silencio al 4 por defecto los
objetivos que un equipo hubiera ajustado. CAPACIDADES_RENOMBRADAS recuerda el
nombre antiguo y capacidadVigente() lo traduce, solo donde el antiguo ya no
existe: en Fiscal la capacidad conserva su nombre y no se toca.

El Excel se edito sustituyendo el texto dentro del .xlsx y no con openpyxl,
que descarta el grafico de la hoja Resumen al guardar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0187ym1kCC8E1LE6XPEyjLRe
</commit_message>
<xml_diff>
--- a/F3M_Tesoreria_assessment_ready_AI_v0.xlsx
+++ b/F3M_Tesoreria_assessment_ready_AI_v0.xlsx
@@ -110,7 +110,7 @@
     <t>Comentarios / hallazgos</t>
   </si>
   <si>
-    <t>Contabilidad y provisión fiscal</t>
+    <t>Control y tratamiento contable</t>
   </si>
   <si>
     <t>1.1 Gobierno contable-fiscal de operaciones de tesorería</t>
@@ -995,7 +995,7 @@
     <t>Dominio</t>
   </si>
   <si>
-    <t>Tesorería: Contabilidad y provisión fiscal, Gestión de riesgos financieros, Mercados de deuda y capitales, Gestión de cash flow y reporte e Inversiones.</t>
+    <t>Tesorería: Control y tratamiento contable, Gestión de riesgos financieros, Mercados de deuda y capitales, Gestión de cash flow y reporte e Inversiones.</t>
   </si>
   <si>
     <t>Escala F3M</t>
@@ -1261,7 +1261,7 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Contabilidad y provisión fiscal</c:v>
+                  <c:v>Control y tratamiento contable</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Gestión de riesgos financieros</c:v>

</xml_diff>